<commit_message>
Deploying to gh-pages from  @ 6bf9a6b732741d7918278275e4262bf159d77c2c 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/15.a.1.1.xlsx
+++ b/en/downloads/data-excel/15.a.1.1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\korozbaeva\Desktop\Показатели ЦУР для Платформы\Национальные показатели ЦУР\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Показатели ЦУР для Платформы\Национальные показатели ЦУР — 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1CD25C-E1EE-4AB2-905A-C4CBB80A8C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -24,18 +25,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
   <si>
     <t>борьбу с загрязнением окружающей среды</t>
   </si>
@@ -116,12 +111,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>15.b.1.1 Объем государственных средств, выделяемых на охрану окружающей среды</t>
-  </si>
-  <si>
-    <t>15.b.1.1 Volume of public funds earmarked for environmental protection</t>
-  </si>
-  <si>
     <t>Көрсөткүчтөрдүн аталышы</t>
   </si>
   <si>
@@ -179,15 +168,22 @@
     <t>(млн.сом)</t>
   </si>
   <si>
-    <t>15.b.1.1 Айлана-чөйрөнү коргоо үчүн бөлүнгөн мамлекеттик акча каражаттарынын көлөмү</t>
+    <t>15.a.1.1 Объем государственных средств, выделяемых на охрану окружающей среды</t>
+  </si>
+  <si>
+    <t>15.a.1.1 Volume of public funds earmarked for environmental protection</t>
+  </si>
+  <si>
+    <t>15.a.1.1 Айлана-чөйрөнү коргоо үчүн бөлүнгөн мамлекеттик акча каражаттарынын көлөмү</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -323,7 +319,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -382,12 +378,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -412,12 +402,21 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Normal 17" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="3"/>
+    <cellStyle name="Normal 17" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 7 2" xfId="2"/>
+    <cellStyle name="Обычный 7 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -694,8 +693,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="37.140625" style="9" customWidth="1"/>
@@ -703,53 +702,54 @@
     <col min="8" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="B1" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="22" t="s">
-        <v>30</v>
+      <c r="C2" s="20" t="s">
+        <v>28</v>
       </c>
       <c r="D2" s="14"/>
       <c r="E2" s="14"/>
       <c r="F2" s="14"/>
       <c r="G2" s="14"/>
     </row>
-    <row r="3" spans="1:17" ht="12.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R3"/>
+    </row>
+    <row r="4" spans="1:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>27</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>29</v>
       </c>
       <c r="D4" s="2">
         <v>2010</v>
@@ -793,16 +793,19 @@
       <c r="Q4" s="1">
         <v>2023</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="24" t="s">
+      <c r="R4" s="1">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>31</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>33</v>
       </c>
       <c r="D5" s="3">
         <v>576.9</v>
@@ -837,19 +840,22 @@
       <c r="N5" s="5">
         <v>588.70000000000005</v>
       </c>
-      <c r="O5" s="27">
+      <c r="O5" s="25">
         <v>689</v>
       </c>
-      <c r="P5" s="27">
+      <c r="P5" s="25">
         <v>1188.7</v>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="25">
         <v>1781</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R5" s="28">
+        <v>3024.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>0</v>
@@ -866,7 +872,7 @@
       <c r="F6" s="18">
         <v>28.2</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="18">
         <v>22.4</v>
       </c>
       <c r="H6" s="6">
@@ -890,19 +896,22 @@
       <c r="N6" s="9">
         <v>62.2</v>
       </c>
-      <c r="O6" s="26">
+      <c r="O6" s="24">
         <v>94.1</v>
       </c>
-      <c r="P6" s="26">
+      <c r="P6" s="24">
         <v>263.89999999999998</v>
       </c>
-      <c r="Q6" s="26">
+      <c r="Q6" s="24">
         <v>409.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R6" s="29">
+        <v>443.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>1</v>
@@ -919,7 +928,7 @@
       <c r="F7" s="18">
         <v>73.2</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="18">
         <v>80.900000000000006</v>
       </c>
       <c r="H7" s="6">
@@ -943,19 +952,22 @@
       <c r="N7" s="9">
         <v>99.4</v>
       </c>
-      <c r="O7" s="26">
+      <c r="O7" s="24">
         <v>147.1</v>
       </c>
-      <c r="P7" s="26">
+      <c r="P7" s="24">
         <v>263.2</v>
       </c>
-      <c r="Q7" s="26">
+      <c r="Q7" s="24">
         <v>435.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R7" s="29">
+        <v>709.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>2</v>
@@ -972,7 +984,7 @@
       <c r="F8" s="18">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="18">
         <v>6.5</v>
       </c>
       <c r="H8" s="6">
@@ -996,19 +1008,22 @@
       <c r="N8" s="9">
         <v>6.1</v>
       </c>
-      <c r="O8" s="26">
+      <c r="O8" s="24">
         <v>10.1</v>
       </c>
-      <c r="P8" s="26">
+      <c r="P8" s="24">
         <v>12.4</v>
       </c>
-      <c r="Q8" s="26">
+      <c r="Q8" s="24">
         <v>27.9</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R8" s="29">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>3</v>
@@ -1025,7 +1040,7 @@
       <c r="F9" s="18">
         <v>1.3</v>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="18">
         <v>1.2</v>
       </c>
       <c r="H9" s="6">
@@ -1045,19 +1060,22 @@
       <c r="N9" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="O9" s="28" t="s">
+      <c r="O9" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="P9" s="28" t="s">
+      <c r="P9" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="Q9" s="28" t="s">
+      <c r="Q9" s="26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R9" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>4</v>
@@ -1074,7 +1092,7 @@
       <c r="F10" s="18">
         <v>26.6</v>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="18">
         <v>63.2</v>
       </c>
       <c r="H10" s="6">
@@ -1095,22 +1113,25 @@
       <c r="M10" s="9">
         <v>64.7</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="24">
         <v>71</v>
       </c>
-      <c r="O10" s="26">
+      <c r="O10" s="24">
         <v>82.1</v>
       </c>
-      <c r="P10" s="26">
+      <c r="P10" s="24">
         <v>93</v>
       </c>
-      <c r="Q10" s="26">
+      <c r="Q10" s="24">
         <v>194.7</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R10" s="29">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>5</v>
@@ -1127,7 +1148,7 @@
       <c r="F11" s="6">
         <v>158.69999999999999</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="6">
         <v>90.9</v>
       </c>
       <c r="H11" s="6">
@@ -1151,19 +1172,22 @@
       <c r="N11" s="9">
         <v>136.30000000000001</v>
       </c>
-      <c r="O11" s="26">
+      <c r="O11" s="24">
         <v>145.30000000000001</v>
       </c>
-      <c r="P11" s="26">
+      <c r="P11" s="24">
         <v>171.5</v>
       </c>
-      <c r="Q11" s="26">
+      <c r="Q11" s="24">
         <v>265.10000000000002</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" ht="24" x14ac:dyDescent="0.25">
+      <c r="R11" s="29">
+        <v>315.10000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="24" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>6</v>
@@ -1180,7 +1204,7 @@
       <c r="F12" s="6">
         <v>29.3</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="6">
         <v>43.9</v>
       </c>
       <c r="H12" s="6">
@@ -1204,19 +1228,22 @@
       <c r="N12" s="9">
         <v>103.3</v>
       </c>
-      <c r="O12" s="26">
+      <c r="O12" s="24">
         <v>98.8</v>
       </c>
-      <c r="P12" s="26">
+      <c r="P12" s="24">
         <v>220.6</v>
       </c>
-      <c r="Q12" s="26">
+      <c r="Q12" s="24">
         <v>193.9</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R12" s="29">
+        <v>238.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>18</v>
@@ -1233,7 +1260,7 @@
       <c r="F13" s="6">
         <v>189.3</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="6">
         <v>235.6</v>
       </c>
       <c r="H13" s="10">
@@ -1257,19 +1284,22 @@
       <c r="N13" s="9">
         <v>103.2</v>
       </c>
-      <c r="O13" s="26">
+      <c r="O13" s="24">
         <v>98.7</v>
       </c>
-      <c r="P13" s="26">
+      <c r="P13" s="24">
         <v>159.30000000000001</v>
       </c>
-      <c r="Q13" s="26">
+      <c r="Q13" s="24">
         <v>251.9</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R13" s="29">
+        <v>1009.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>16</v>
@@ -1286,7 +1316,7 @@
       <c r="F14" s="6">
         <v>4.5999999999999996</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="6">
         <v>6.2</v>
       </c>
       <c r="H14" s="10">
@@ -1310,19 +1340,22 @@
       <c r="N14" s="9">
         <v>1.8</v>
       </c>
-      <c r="O14" s="26">
+      <c r="O14" s="24">
         <v>1.8</v>
       </c>
-      <c r="P14" s="26">
+      <c r="P14" s="24">
         <v>1.7</v>
       </c>
-      <c r="Q14" s="26">
+      <c r="Q14" s="24">
         <v>1.7</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R14" s="29">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>17</v>
@@ -1330,16 +1363,16 @@
       <c r="C15" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="6">
         <v>11</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="6">
         <v>11.2</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="6">
         <v>9.8000000000000007</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="6">
         <v>11.2</v>
       </c>
       <c r="H15" s="9">
@@ -1363,19 +1396,22 @@
       <c r="N15" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="O15" s="28" t="s">
+      <c r="O15" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="P15" s="28" t="s">
+      <c r="P15" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="Q15" s="28" t="s">
+      <c r="Q15" s="26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R15" s="29">
+        <v>19.8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>7</v>
@@ -1416,14 +1452,17 @@
       <c r="N16" s="12">
         <v>5.4</v>
       </c>
-      <c r="O16" s="29">
+      <c r="O16" s="27">
         <v>10.9</v>
       </c>
-      <c r="P16" s="29">
+      <c r="P16" s="27">
         <v>3.1</v>
       </c>
-      <c r="Q16" s="29">
+      <c r="Q16" s="27">
         <v>1.5</v>
+      </c>
+      <c r="R16" s="30">
+        <v>0.7</v>
       </c>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.25">

</xml_diff>